<commit_message>
Merge WK1ST+WK2ND on Fridays; correct 2026-09-18 report
Per sirichai: on a Friday report date, WK1ST would only span Fri-Sun
(3 days) - too short to be meaningful standalone, so WK1ST's upper bound
extends through the following Sunday (both weeks combined) and WK2ND's
booking figures come out blank (already counted in WK1ST above). Applies
to any report_date.weekday() == 4, not just this one Friday.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock Daily 2026-09-18.xlsx
+++ b/Stock Daily 2026-09-18.xlsx
@@ -1685,24 +1685,27 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="22" fillId="10" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1736,6 +1739,9 @@
     <xf numFmtId="165" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="24" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1752,12 +1758,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="10" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4000,7 +4000,7 @@
       <c r="H29" s="188" t="n"/>
       <c r="I29" s="196" t="inlineStr">
         <is>
-          <t>18-20/09/2026</t>
+          <t>18-27/09/2026</t>
         </is>
       </c>
       <c r="J29" s="187" t="n"/>
@@ -4037,7 +4037,7 @@
       <c r="AC29" s="188" t="n"/>
       <c r="AD29" s="196" t="inlineStr">
         <is>
-          <t>18-20/09/2026</t>
+          <t>18-27/09/2026</t>
         </is>
       </c>
       <c r="AE29" s="187" t="n"/>
@@ -4255,11 +4255,11 @@
         </is>
       </c>
       <c r="C31" s="206" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D31" s="207" t="n"/>
       <c r="E31" s="207" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="F31" s="207" t="n"/>
       <c r="G31" s="207" t="n"/>
@@ -4322,7 +4322,7 @@
       <c r="AD31" s="229" t="n"/>
       <c r="AE31" s="229" t="n"/>
       <c r="AF31" s="230" t="n"/>
-      <c r="AG31" s="225">
+      <c r="AG31" s="231">
         <f>SUM(AG4-X31)</f>
         <v/>
       </c>
@@ -4374,46 +4374,48 @@
         <v>2</v>
       </c>
       <c r="D32" s="215" t="n"/>
-      <c r="E32" s="215" t="n"/>
+      <c r="E32" s="215" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" s="215" t="n"/>
       <c r="G32" s="215" t="n"/>
       <c r="H32" s="215" t="n"/>
       <c r="I32" s="215" t="n"/>
       <c r="J32" s="215" t="n"/>
       <c r="K32" s="216" t="n"/>
-      <c r="L32" s="231">
+      <c r="L32" s="232">
         <f>SUM(L5-C32)</f>
         <v/>
       </c>
-      <c r="M32" s="232">
+      <c r="M32" s="233">
         <f>SUM(M5-D32)</f>
         <v/>
       </c>
-      <c r="N32" s="232">
+      <c r="N32" s="233">
         <f>SUM(N5-E32)</f>
         <v/>
       </c>
-      <c r="O32" s="232">
+      <c r="O32" s="233">
         <f>SUM(O5-F32)</f>
         <v/>
       </c>
-      <c r="P32" s="232">
+      <c r="P32" s="233">
         <f>SUM(P5-G32)</f>
         <v/>
       </c>
-      <c r="Q32" s="232">
+      <c r="Q32" s="233">
         <f>SUM(Q5-H32)</f>
         <v/>
       </c>
-      <c r="R32" s="232">
+      <c r="R32" s="233">
         <f>SUM(R5-I32)</f>
         <v/>
       </c>
-      <c r="S32" s="232">
+      <c r="S32" s="233">
         <f>SUM(S5-J32)</f>
         <v/>
       </c>
-      <c r="T32" s="233">
+      <c r="T32" s="234">
         <f>SUM(T5-K32)</f>
         <v/>
       </c>
@@ -4427,48 +4429,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X32" s="234" t="n"/>
-      <c r="Y32" s="235" t="n"/>
-      <c r="Z32" s="235" t="n"/>
-      <c r="AA32" s="235" t="n"/>
-      <c r="AB32" s="235" t="n"/>
-      <c r="AC32" s="235" t="n"/>
-      <c r="AD32" s="235" t="n"/>
-      <c r="AE32" s="235" t="n"/>
-      <c r="AF32" s="236" t="n"/>
-      <c r="AG32" s="231">
+      <c r="X32" s="235" t="n"/>
+      <c r="Y32" s="236" t="n"/>
+      <c r="Z32" s="236" t="n"/>
+      <c r="AA32" s="236" t="n"/>
+      <c r="AB32" s="236" t="n"/>
+      <c r="AC32" s="236" t="n"/>
+      <c r="AD32" s="236" t="n"/>
+      <c r="AE32" s="236" t="n"/>
+      <c r="AF32" s="237" t="n"/>
+      <c r="AG32" s="232">
         <f>SUM(AG5-X32)</f>
         <v/>
       </c>
-      <c r="AH32" s="232">
+      <c r="AH32" s="233">
         <f>SUM(AH5-Y32)</f>
         <v/>
       </c>
-      <c r="AI32" s="232">
+      <c r="AI32" s="233">
         <f>SUM(AI5-Z32)</f>
         <v/>
       </c>
-      <c r="AJ32" s="232">
+      <c r="AJ32" s="233">
         <f>SUM(AJ5-AA32)</f>
         <v/>
       </c>
-      <c r="AK32" s="232">
+      <c r="AK32" s="233">
         <f>SUM(AK5-AB32)</f>
         <v/>
       </c>
-      <c r="AL32" s="232">
+      <c r="AL32" s="233">
         <f>SUM(AL5-AC32)</f>
         <v/>
       </c>
-      <c r="AM32" s="232">
+      <c r="AM32" s="233">
         <f>SUM(AM5-AD32)</f>
         <v/>
       </c>
-      <c r="AN32" s="232">
+      <c r="AN32" s="233">
         <f>SUM(AN5-AE32)</f>
         <v/>
       </c>
-      <c r="AO32" s="233">
+      <c r="AO32" s="234">
         <f>SUM(AO5-AF32)</f>
         <v/>
       </c>
@@ -4493,39 +4495,39 @@
       <c r="I33" s="215" t="n"/>
       <c r="J33" s="215" t="n"/>
       <c r="K33" s="216" t="n"/>
-      <c r="L33" s="231">
+      <c r="L33" s="232">
         <f>SUM(L6-C33)</f>
         <v/>
       </c>
-      <c r="M33" s="232">
+      <c r="M33" s="233">
         <f>SUM(M6-D33)</f>
         <v/>
       </c>
-      <c r="N33" s="232">
+      <c r="N33" s="233">
         <f>SUM(N6-E33)</f>
         <v/>
       </c>
-      <c r="O33" s="232">
+      <c r="O33" s="233">
         <f>SUM(O6-F33)</f>
         <v/>
       </c>
-      <c r="P33" s="232">
+      <c r="P33" s="233">
         <f>SUM(P6-G33)</f>
         <v/>
       </c>
-      <c r="Q33" s="232">
+      <c r="Q33" s="233">
         <f>SUM(Q6-H33)</f>
         <v/>
       </c>
-      <c r="R33" s="232">
+      <c r="R33" s="233">
         <f>SUM(R6-I33)</f>
         <v/>
       </c>
-      <c r="S33" s="232">
+      <c r="S33" s="233">
         <f>SUM(S6-J33)</f>
         <v/>
       </c>
-      <c r="T33" s="233">
+      <c r="T33" s="234">
         <f>SUM(T6-K33)</f>
         <v/>
       </c>
@@ -4539,48 +4541,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X33" s="234" t="n"/>
-      <c r="Y33" s="235" t="n"/>
-      <c r="Z33" s="235" t="n"/>
-      <c r="AA33" s="235" t="n"/>
-      <c r="AB33" s="235" t="n"/>
-      <c r="AC33" s="235" t="n"/>
-      <c r="AD33" s="235" t="n"/>
-      <c r="AE33" s="235" t="n"/>
-      <c r="AF33" s="236" t="n"/>
-      <c r="AG33" s="231">
+      <c r="X33" s="235" t="n"/>
+      <c r="Y33" s="236" t="n"/>
+      <c r="Z33" s="236" t="n"/>
+      <c r="AA33" s="236" t="n"/>
+      <c r="AB33" s="236" t="n"/>
+      <c r="AC33" s="236" t="n"/>
+      <c r="AD33" s="236" t="n"/>
+      <c r="AE33" s="236" t="n"/>
+      <c r="AF33" s="237" t="n"/>
+      <c r="AG33" s="232">
         <f>SUM(AG6-X33)</f>
         <v/>
       </c>
-      <c r="AH33" s="232">
+      <c r="AH33" s="233">
         <f>SUM(AH6-Y33)</f>
         <v/>
       </c>
-      <c r="AI33" s="232">
+      <c r="AI33" s="233">
         <f>SUM(AI6-Z33)</f>
         <v/>
       </c>
-      <c r="AJ33" s="232">
+      <c r="AJ33" s="233">
         <f>SUM(AJ6-AA33)</f>
         <v/>
       </c>
-      <c r="AK33" s="232">
+      <c r="AK33" s="233">
         <f>SUM(AK6-AB33)</f>
         <v/>
       </c>
-      <c r="AL33" s="232">
+      <c r="AL33" s="233">
         <f>SUM(AL6-AC33)</f>
         <v/>
       </c>
-      <c r="AM33" s="232">
+      <c r="AM33" s="233">
         <f>SUM(AM6-AD33)</f>
         <v/>
       </c>
-      <c r="AN33" s="232">
+      <c r="AN33" s="233">
         <f>SUM(AN6-AE33)</f>
         <v/>
       </c>
-      <c r="AO33" s="233">
+      <c r="AO33" s="234">
         <f>SUM(AO6-AF33)</f>
         <v/>
       </c>
@@ -4596,48 +4598,48 @@
           <t>ICD</t>
         </is>
       </c>
-      <c r="C34" s="234" t="n"/>
-      <c r="D34" s="235" t="n"/>
-      <c r="E34" s="235" t="n"/>
-      <c r="F34" s="235" t="n"/>
-      <c r="G34" s="235" t="n"/>
-      <c r="H34" s="235" t="n"/>
-      <c r="I34" s="235" t="n"/>
-      <c r="J34" s="235" t="n"/>
-      <c r="K34" s="236" t="n"/>
-      <c r="L34" s="231">
+      <c r="C34" s="235" t="n"/>
+      <c r="D34" s="236" t="n"/>
+      <c r="E34" s="236" t="n"/>
+      <c r="F34" s="236" t="n"/>
+      <c r="G34" s="236" t="n"/>
+      <c r="H34" s="236" t="n"/>
+      <c r="I34" s="236" t="n"/>
+      <c r="J34" s="236" t="n"/>
+      <c r="K34" s="237" t="n"/>
+      <c r="L34" s="232">
         <f>SUM(L7-C34)</f>
         <v/>
       </c>
-      <c r="M34" s="232">
+      <c r="M34" s="233">
         <f>SUM(M7-D34)</f>
         <v/>
       </c>
-      <c r="N34" s="232">
+      <c r="N34" s="233">
         <f>SUM(N7-E34)</f>
         <v/>
       </c>
-      <c r="O34" s="232">
+      <c r="O34" s="233">
         <f>SUM(O7-F34)</f>
         <v/>
       </c>
-      <c r="P34" s="232">
+      <c r="P34" s="233">
         <f>SUM(P7-G34)</f>
         <v/>
       </c>
-      <c r="Q34" s="232">
+      <c r="Q34" s="233">
         <f>SUM(Q7-H34)</f>
         <v/>
       </c>
-      <c r="R34" s="232">
+      <c r="R34" s="233">
         <f>SUM(R7-I34)</f>
         <v/>
       </c>
-      <c r="S34" s="232">
+      <c r="S34" s="233">
         <f>SUM(S7-J34)</f>
         <v/>
       </c>
-      <c r="T34" s="233">
+      <c r="T34" s="234">
         <f>SUM(T7-K34)</f>
         <v/>
       </c>
@@ -4651,48 +4653,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X34" s="234" t="n"/>
-      <c r="Y34" s="235" t="n"/>
-      <c r="Z34" s="235" t="n"/>
-      <c r="AA34" s="235" t="n"/>
-      <c r="AB34" s="235" t="n"/>
-      <c r="AC34" s="235" t="n"/>
-      <c r="AD34" s="235" t="n"/>
-      <c r="AE34" s="235" t="n"/>
-      <c r="AF34" s="236" t="n"/>
-      <c r="AG34" s="231">
+      <c r="X34" s="235" t="n"/>
+      <c r="Y34" s="236" t="n"/>
+      <c r="Z34" s="236" t="n"/>
+      <c r="AA34" s="236" t="n"/>
+      <c r="AB34" s="236" t="n"/>
+      <c r="AC34" s="236" t="n"/>
+      <c r="AD34" s="236" t="n"/>
+      <c r="AE34" s="236" t="n"/>
+      <c r="AF34" s="237" t="n"/>
+      <c r="AG34" s="232">
         <f>SUM(AG7-X34)</f>
         <v/>
       </c>
-      <c r="AH34" s="232">
+      <c r="AH34" s="233">
         <f>SUM(AH7-Y34)</f>
         <v/>
       </c>
-      <c r="AI34" s="232">
+      <c r="AI34" s="233">
         <f>SUM(AI7-Z34)</f>
         <v/>
       </c>
-      <c r="AJ34" s="232">
+      <c r="AJ34" s="233">
         <f>SUM(AJ7-AA34)</f>
         <v/>
       </c>
-      <c r="AK34" s="232">
+      <c r="AK34" s="233">
         <f>SUM(AK7-AB34)</f>
         <v/>
       </c>
-      <c r="AL34" s="232">
+      <c r="AL34" s="233">
         <f>SUM(AL7-AC34)</f>
         <v/>
       </c>
-      <c r="AM34" s="232">
+      <c r="AM34" s="233">
         <f>SUM(AM7-AD34)</f>
         <v/>
       </c>
-      <c r="AN34" s="232">
+      <c r="AN34" s="233">
         <f>SUM(AN7-AE34)</f>
         <v/>
       </c>
-      <c r="AO34" s="233">
+      <c r="AO34" s="234">
         <f>SUM(AO7-AF34)</f>
         <v/>
       </c>
@@ -4708,52 +4710,52 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C35" s="237" t="n">
-        <v>94</v>
+      <c r="C35" s="238" t="n">
+        <v>204</v>
       </c>
       <c r="D35" s="223" t="n"/>
       <c r="E35" s="223" t="n">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="F35" s="223" t="n"/>
       <c r="G35" s="223" t="n"/>
       <c r="H35" s="223" t="n"/>
       <c r="I35" s="223" t="n"/>
       <c r="J35" s="223" t="n"/>
-      <c r="K35" s="238" t="n"/>
-      <c r="L35" s="239">
+      <c r="K35" s="239" t="n"/>
+      <c r="L35" s="240">
         <f>SUM(L8-C35)</f>
         <v/>
       </c>
-      <c r="M35" s="240">
+      <c r="M35" s="241">
         <f>SUM(M8-D35)</f>
         <v/>
       </c>
-      <c r="N35" s="240">
+      <c r="N35" s="241">
         <f>SUM(N8-E35)</f>
         <v/>
       </c>
-      <c r="O35" s="240">
+      <c r="O35" s="241">
         <f>SUM(O8-F35)</f>
         <v/>
       </c>
-      <c r="P35" s="240">
+      <c r="P35" s="241">
         <f>SUM(P8-G35)</f>
         <v/>
       </c>
-      <c r="Q35" s="240">
+      <c r="Q35" s="241">
         <f>SUM(Q8-H35)</f>
         <v/>
       </c>
-      <c r="R35" s="240">
+      <c r="R35" s="241">
         <f>SUM(R8-I35)</f>
         <v/>
       </c>
-      <c r="S35" s="240">
+      <c r="S35" s="241">
         <f>SUM(S8-J35)</f>
         <v/>
       </c>
-      <c r="T35" s="241">
+      <c r="T35" s="242">
         <f>SUM(T8-K35)</f>
         <v/>
       </c>
@@ -4767,54 +4769,56 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X35" s="237" t="n">
-        <v>54</v>
+      <c r="X35" s="238" t="n">
+        <v>155</v>
       </c>
       <c r="Y35" s="223" t="n"/>
       <c r="Z35" s="223" t="n">
-        <v>36</v>
-      </c>
-      <c r="AA35" s="223" t="n"/>
+        <v>119</v>
+      </c>
+      <c r="AA35" s="223" t="n">
+        <v>2</v>
+      </c>
       <c r="AB35" s="223" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="AC35" s="223" t="n"/>
       <c r="AD35" s="223" t="n"/>
       <c r="AE35" s="223" t="n"/>
-      <c r="AF35" s="238" t="n"/>
-      <c r="AG35" s="239">
+      <c r="AF35" s="239" t="n"/>
+      <c r="AG35" s="240">
         <f>SUM(AG8-X35)</f>
         <v/>
       </c>
-      <c r="AH35" s="240">
+      <c r="AH35" s="241">
         <f>SUM(AH8-Y35)</f>
         <v/>
       </c>
-      <c r="AI35" s="240">
+      <c r="AI35" s="241">
         <f>SUM(AI8-Z35)</f>
         <v/>
       </c>
-      <c r="AJ35" s="240">
+      <c r="AJ35" s="241">
         <f>SUM(AJ8-AA35)</f>
         <v/>
       </c>
-      <c r="AK35" s="240">
+      <c r="AK35" s="241">
         <f>SUM(AK8-AB35)</f>
         <v/>
       </c>
-      <c r="AL35" s="240">
+      <c r="AL35" s="241">
         <f>SUM(AL8-AC35)</f>
         <v/>
       </c>
-      <c r="AM35" s="240">
+      <c r="AM35" s="241">
         <f>SUM(AM8-AD35)</f>
         <v/>
       </c>
-      <c r="AN35" s="240">
+      <c r="AN35" s="241">
         <f>SUM(AN8-AE35)</f>
         <v/>
       </c>
-      <c r="AO35" s="241">
+      <c r="AO35" s="242">
         <f>SUM(AO8-AF35)</f>
         <v/>
       </c>
@@ -4830,56 +4834,58 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C36" s="237" t="n">
-        <v>123</v>
-      </c>
-      <c r="D36" s="223" t="n"/>
+      <c r="C36" s="238" t="n">
+        <v>274</v>
+      </c>
+      <c r="D36" s="223" t="n">
+        <v>1</v>
+      </c>
       <c r="E36" s="223" t="n">
-        <v>59</v>
+        <v>204</v>
       </c>
       <c r="F36" s="223" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G36" s="223" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="H36" s="223" t="n"/>
       <c r="I36" s="223" t="n"/>
       <c r="J36" s="223" t="n"/>
-      <c r="K36" s="238" t="n"/>
-      <c r="L36" s="239">
+      <c r="K36" s="239" t="n"/>
+      <c r="L36" s="240">
         <f>SUM(L9-C36)</f>
         <v/>
       </c>
-      <c r="M36" s="240">
+      <c r="M36" s="241">
         <f>SUM(M9-D36)</f>
         <v/>
       </c>
-      <c r="N36" s="240">
+      <c r="N36" s="241">
         <f>SUM(N9-E36)</f>
         <v/>
       </c>
-      <c r="O36" s="240">
+      <c r="O36" s="241">
         <f>SUM(O9-F36)</f>
         <v/>
       </c>
-      <c r="P36" s="240">
+      <c r="P36" s="243">
         <f>SUM(P9-G36)</f>
         <v/>
       </c>
-      <c r="Q36" s="240">
+      <c r="Q36" s="241">
         <f>SUM(Q9-H36)</f>
         <v/>
       </c>
-      <c r="R36" s="240">
+      <c r="R36" s="241">
         <f>SUM(R9-I36)</f>
         <v/>
       </c>
-      <c r="S36" s="240">
+      <c r="S36" s="241">
         <f>SUM(S9-J36)</f>
         <v/>
       </c>
-      <c r="T36" s="241">
+      <c r="T36" s="242">
         <f>SUM(T9-K36)</f>
         <v/>
       </c>
@@ -4893,52 +4899,52 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X36" s="237" t="n">
-        <v>3</v>
+      <c r="X36" s="238" t="n">
+        <v>14</v>
       </c>
       <c r="Y36" s="223" t="n"/>
       <c r="Z36" s="223" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="AA36" s="223" t="n"/>
       <c r="AB36" s="223" t="n"/>
       <c r="AC36" s="223" t="n"/>
       <c r="AD36" s="223" t="n"/>
       <c r="AE36" s="223" t="n"/>
-      <c r="AF36" s="238" t="n"/>
-      <c r="AG36" s="239">
+      <c r="AF36" s="239" t="n"/>
+      <c r="AG36" s="240">
         <f>SUM(AG9-X36)</f>
         <v/>
       </c>
-      <c r="AH36" s="240">
+      <c r="AH36" s="241">
         <f>SUM(AH9-Y36)</f>
         <v/>
       </c>
-      <c r="AI36" s="240">
+      <c r="AI36" s="241">
         <f>SUM(AI9-Z36)</f>
         <v/>
       </c>
-      <c r="AJ36" s="240">
+      <c r="AJ36" s="241">
         <f>SUM(AJ9-AA36)</f>
         <v/>
       </c>
-      <c r="AK36" s="240">
+      <c r="AK36" s="241">
         <f>SUM(AK9-AB36)</f>
         <v/>
       </c>
-      <c r="AL36" s="240">
+      <c r="AL36" s="241">
         <f>SUM(AL9-AC36)</f>
         <v/>
       </c>
-      <c r="AM36" s="240">
+      <c r="AM36" s="241">
         <f>SUM(AM9-AD36)</f>
         <v/>
       </c>
-      <c r="AN36" s="240">
+      <c r="AN36" s="241">
         <f>SUM(AN9-AE36)</f>
         <v/>
       </c>
-      <c r="AO36" s="241">
+      <c r="AO36" s="242">
         <f>SUM(AO9-AF36)</f>
         <v/>
       </c>
@@ -4955,39 +4961,39 @@
       <c r="I37" s="49" t="n"/>
       <c r="J37" s="49" t="n"/>
       <c r="K37" s="82" t="n"/>
-      <c r="L37" s="242">
+      <c r="L37" s="244">
         <f>SUM(L10-C37)</f>
         <v/>
       </c>
-      <c r="M37" s="243">
+      <c r="M37" s="245">
         <f>SUM(M10-D37)</f>
         <v/>
       </c>
-      <c r="N37" s="243">
+      <c r="N37" s="245">
         <f>SUM(N10-E37)</f>
         <v/>
       </c>
-      <c r="O37" s="243">
+      <c r="O37" s="245">
         <f>SUM(O10-F37)</f>
         <v/>
       </c>
-      <c r="P37" s="243">
+      <c r="P37" s="245">
         <f>SUM(P10-G37)</f>
         <v/>
       </c>
-      <c r="Q37" s="243">
+      <c r="Q37" s="245">
         <f>SUM(Q10-H37)</f>
         <v/>
       </c>
-      <c r="R37" s="243">
+      <c r="R37" s="245">
         <f>SUM(R10-I37)</f>
         <v/>
       </c>
-      <c r="S37" s="243">
+      <c r="S37" s="245">
         <f>SUM(S10-J37)</f>
         <v/>
       </c>
-      <c r="T37" s="244">
+      <c r="T37" s="246">
         <f>SUM(T10-K37)</f>
         <v/>
       </c>
@@ -5001,52 +5007,52 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X37" s="237" t="n">
-        <v>118</v>
+      <c r="X37" s="238" t="n">
+        <v>311</v>
       </c>
       <c r="Y37" s="223" t="n"/>
       <c r="Z37" s="223" t="n">
-        <v>148</v>
+        <v>338</v>
       </c>
       <c r="AA37" s="223" t="n"/>
       <c r="AB37" s="223" t="n"/>
       <c r="AC37" s="223" t="n"/>
       <c r="AD37" s="223" t="n"/>
       <c r="AE37" s="223" t="n"/>
-      <c r="AF37" s="238" t="n"/>
-      <c r="AG37" s="239">
+      <c r="AF37" s="239" t="n"/>
+      <c r="AG37" s="240">
         <f>SUM(AG10-X37)</f>
         <v/>
       </c>
-      <c r="AH37" s="240">
+      <c r="AH37" s="241">
         <f>SUM(AH10-Y37)</f>
         <v/>
       </c>
-      <c r="AI37" s="240">
+      <c r="AI37" s="241">
         <f>SUM(AI10-Z37)</f>
         <v/>
       </c>
-      <c r="AJ37" s="240">
+      <c r="AJ37" s="241">
         <f>SUM(AJ10-AA37)</f>
         <v/>
       </c>
-      <c r="AK37" s="240">
+      <c r="AK37" s="241">
         <f>SUM(AK10-AB37)</f>
         <v/>
       </c>
-      <c r="AL37" s="240">
+      <c r="AL37" s="241">
         <f>SUM(AL10-AC37)</f>
         <v/>
       </c>
-      <c r="AM37" s="240">
+      <c r="AM37" s="241">
         <f>SUM(AM10-AD37)</f>
         <v/>
       </c>
-      <c r="AN37" s="240">
+      <c r="AN37" s="241">
         <f>SUM(AN10-AE37)</f>
         <v/>
       </c>
-      <c r="AO37" s="241">
+      <c r="AO37" s="242">
         <f>SUM(AO10-AF37)</f>
         <v/>
       </c>
@@ -5063,39 +5069,39 @@
       <c r="I38" s="49" t="n"/>
       <c r="J38" s="49" t="n"/>
       <c r="K38" s="82" t="n"/>
-      <c r="L38" s="242">
+      <c r="L38" s="244">
         <f>SUM(L11-C38)</f>
         <v/>
       </c>
-      <c r="M38" s="243">
+      <c r="M38" s="245">
         <f>SUM(M11-D38)</f>
         <v/>
       </c>
-      <c r="N38" s="243">
+      <c r="N38" s="245">
         <f>SUM(N11-E38)</f>
         <v/>
       </c>
-      <c r="O38" s="243">
+      <c r="O38" s="245">
         <f>SUM(O11-F38)</f>
         <v/>
       </c>
-      <c r="P38" s="243">
+      <c r="P38" s="245">
         <f>SUM(P11-G38)</f>
         <v/>
       </c>
-      <c r="Q38" s="243">
+      <c r="Q38" s="245">
         <f>SUM(Q11-H38)</f>
         <v/>
       </c>
-      <c r="R38" s="243">
+      <c r="R38" s="245">
         <f>SUM(R11-I38)</f>
         <v/>
       </c>
-      <c r="S38" s="243">
+      <c r="S38" s="245">
         <f>SUM(S11-J38)</f>
         <v/>
       </c>
-      <c r="T38" s="244">
+      <c r="T38" s="246">
         <f>SUM(T11-K38)</f>
         <v/>
       </c>
@@ -5110,39 +5116,39 @@
       <c r="AD38" s="49" t="n"/>
       <c r="AE38" s="49" t="n"/>
       <c r="AF38" s="82" t="n"/>
-      <c r="AG38" s="242">
+      <c r="AG38" s="244">
         <f>SUM(AG11-X38)</f>
         <v/>
       </c>
-      <c r="AH38" s="243">
+      <c r="AH38" s="245">
         <f>SUM(AH11-Y38)</f>
         <v/>
       </c>
-      <c r="AI38" s="243">
+      <c r="AI38" s="245">
         <f>SUM(AI11-Z38)</f>
         <v/>
       </c>
-      <c r="AJ38" s="243">
+      <c r="AJ38" s="245">
         <f>SUM(AJ11-AA38)</f>
         <v/>
       </c>
-      <c r="AK38" s="243">
+      <c r="AK38" s="245">
         <f>SUM(AK11-AB38)</f>
         <v/>
       </c>
-      <c r="AL38" s="243">
+      <c r="AL38" s="245">
         <f>SUM(AL11-AC38)</f>
         <v/>
       </c>
-      <c r="AM38" s="243">
+      <c r="AM38" s="245">
         <f>SUM(AM11-AD38)</f>
         <v/>
       </c>
-      <c r="AN38" s="243">
+      <c r="AN38" s="245">
         <f>SUM(AN11-AE38)</f>
         <v/>
       </c>
-      <c r="AO38" s="244">
+      <c r="AO38" s="246">
         <f>SUM(AO11-AF38)</f>
         <v/>
       </c>
@@ -5159,39 +5165,39 @@
       <c r="I39" s="49" t="n"/>
       <c r="J39" s="49" t="n"/>
       <c r="K39" s="82" t="n"/>
-      <c r="L39" s="242">
+      <c r="L39" s="244">
         <f>SUM(L12-C39)</f>
         <v/>
       </c>
-      <c r="M39" s="243">
+      <c r="M39" s="245">
         <f>SUM(M12-D39)</f>
         <v/>
       </c>
-      <c r="N39" s="243">
+      <c r="N39" s="245">
         <f>SUM(N12-E39)</f>
         <v/>
       </c>
-      <c r="O39" s="243">
+      <c r="O39" s="245">
         <f>SUM(O12-F39)</f>
         <v/>
       </c>
-      <c r="P39" s="243">
+      <c r="P39" s="245">
         <f>SUM(P12-G39)</f>
         <v/>
       </c>
-      <c r="Q39" s="243">
+      <c r="Q39" s="245">
         <f>SUM(Q12-H39)</f>
         <v/>
       </c>
-      <c r="R39" s="243">
+      <c r="R39" s="245">
         <f>SUM(R12-I39)</f>
         <v/>
       </c>
-      <c r="S39" s="243">
+      <c r="S39" s="245">
         <f>SUM(S12-J39)</f>
         <v/>
       </c>
-      <c r="T39" s="244">
+      <c r="T39" s="246">
         <f>SUM(T12-K39)</f>
         <v/>
       </c>
@@ -5206,39 +5212,39 @@
       <c r="AD39" s="49" t="n"/>
       <c r="AE39" s="49" t="n"/>
       <c r="AF39" s="82" t="n"/>
-      <c r="AG39" s="242">
+      <c r="AG39" s="244">
         <f>SUM(AG12-X39)</f>
         <v/>
       </c>
-      <c r="AH39" s="243">
+      <c r="AH39" s="245">
         <f>SUM(AH12-Y39)</f>
         <v/>
       </c>
-      <c r="AI39" s="243">
+      <c r="AI39" s="245">
         <f>SUM(AI12-Z39)</f>
         <v/>
       </c>
-      <c r="AJ39" s="243">
+      <c r="AJ39" s="245">
         <f>SUM(AJ12-AA39)</f>
         <v/>
       </c>
-      <c r="AK39" s="243">
+      <c r="AK39" s="245">
         <f>SUM(AK12-AB39)</f>
         <v/>
       </c>
-      <c r="AL39" s="243">
+      <c r="AL39" s="245">
         <f>SUM(AL12-AC39)</f>
         <v/>
       </c>
-      <c r="AM39" s="243">
+      <c r="AM39" s="245">
         <f>SUM(AM12-AD39)</f>
         <v/>
       </c>
-      <c r="AN39" s="243">
+      <c r="AN39" s="245">
         <f>SUM(AN12-AE39)</f>
         <v/>
       </c>
-      <c r="AO39" s="244">
+      <c r="AO39" s="246">
         <f>SUM(AO12-AF39)</f>
         <v/>
       </c>
@@ -5264,39 +5270,39 @@
       <c r="I40" s="85" t="n"/>
       <c r="J40" s="85" t="n"/>
       <c r="K40" s="86" t="n"/>
-      <c r="L40" s="245">
+      <c r="L40" s="247">
         <f>SUM(L13-C40)</f>
         <v/>
       </c>
-      <c r="M40" s="246">
+      <c r="M40" s="248">
         <f>SUM(M13-D40)</f>
         <v/>
       </c>
-      <c r="N40" s="246">
+      <c r="N40" s="248">
         <f>SUM(N13-E40)</f>
         <v/>
       </c>
-      <c r="O40" s="246">
+      <c r="O40" s="248">
         <f>SUM(O13-F40)</f>
         <v/>
       </c>
-      <c r="P40" s="246">
+      <c r="P40" s="248">
         <f>SUM(P13-G40)</f>
         <v/>
       </c>
-      <c r="Q40" s="246">
+      <c r="Q40" s="248">
         <f>SUM(Q13-H40)</f>
         <v/>
       </c>
-      <c r="R40" s="246">
+      <c r="R40" s="248">
         <f>SUM(R13-I40)</f>
         <v/>
       </c>
-      <c r="S40" s="246">
+      <c r="S40" s="248">
         <f>SUM(S13-J40)</f>
         <v/>
       </c>
-      <c r="T40" s="247">
+      <c r="T40" s="249">
         <f>SUM(T13-K40)</f>
         <v/>
       </c>
@@ -5315,39 +5321,39 @@
       <c r="AD40" s="85" t="n"/>
       <c r="AE40" s="85" t="n"/>
       <c r="AF40" s="86" t="n"/>
-      <c r="AG40" s="242">
+      <c r="AG40" s="244">
         <f>SUM(AG13-X40)</f>
         <v/>
       </c>
-      <c r="AH40" s="243">
+      <c r="AH40" s="245">
         <f>SUM(AH13-Y40)</f>
         <v/>
       </c>
-      <c r="AI40" s="243">
+      <c r="AI40" s="245">
         <f>SUM(AI13-Z40)</f>
         <v/>
       </c>
-      <c r="AJ40" s="243">
+      <c r="AJ40" s="245">
         <f>SUM(AJ13-AA40)</f>
         <v/>
       </c>
-      <c r="AK40" s="243">
+      <c r="AK40" s="245">
         <f>SUM(AK13-AB40)</f>
         <v/>
       </c>
-      <c r="AL40" s="243">
+      <c r="AL40" s="245">
         <f>SUM(AL13-AC40)</f>
         <v/>
       </c>
-      <c r="AM40" s="243">
+      <c r="AM40" s="245">
         <f>SUM(AM13-AD40)</f>
         <v/>
       </c>
-      <c r="AN40" s="243">
+      <c r="AN40" s="245">
         <f>SUM(AN13-AE40)</f>
         <v/>
       </c>
-      <c r="AO40" s="244">
+      <c r="AO40" s="246">
         <f>SUM(AO13-AF40)</f>
         <v/>
       </c>
@@ -5784,20 +5790,16 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="C45" s="206" t="n">
-        <v>13</v>
-      </c>
+      <c r="C45" s="206" t="n"/>
       <c r="D45" s="207" t="n"/>
-      <c r="E45" s="207" t="n">
-        <v>19</v>
-      </c>
+      <c r="E45" s="207" t="n"/>
       <c r="F45" s="207" t="n"/>
       <c r="G45" s="207" t="n"/>
       <c r="H45" s="207" t="n"/>
       <c r="I45" s="207" t="n"/>
       <c r="J45" s="207" t="n"/>
       <c r="K45" s="208" t="n"/>
-      <c r="L45" s="248">
+      <c r="L45" s="225">
         <f>SUM(L31-C45)</f>
         <v/>
       </c>
@@ -5852,7 +5854,7 @@
       <c r="AD45" s="229" t="n"/>
       <c r="AE45" s="229" t="n"/>
       <c r="AF45" s="230" t="n"/>
-      <c r="AG45" s="225">
+      <c r="AG45" s="231">
         <f>SUM(AG31-X45)</f>
         <v/>
       </c>
@@ -5902,48 +5904,46 @@
       </c>
       <c r="C46" s="214" t="n"/>
       <c r="D46" s="215" t="n"/>
-      <c r="E46" s="215" t="n">
-        <v>1</v>
-      </c>
+      <c r="E46" s="215" t="n"/>
       <c r="F46" s="215" t="n"/>
       <c r="G46" s="215" t="n"/>
       <c r="H46" s="215" t="n"/>
       <c r="I46" s="215" t="n"/>
       <c r="J46" s="215" t="n"/>
       <c r="K46" s="216" t="n"/>
-      <c r="L46" s="231">
+      <c r="L46" s="232">
         <f>SUM(L32-C46)</f>
         <v/>
       </c>
-      <c r="M46" s="232">
+      <c r="M46" s="233">
         <f>SUM(M32-D46)</f>
         <v/>
       </c>
-      <c r="N46" s="232">
+      <c r="N46" s="233">
         <f>SUM(N32-E46)</f>
         <v/>
       </c>
-      <c r="O46" s="232">
+      <c r="O46" s="233">
         <f>SUM(O32-F46)</f>
         <v/>
       </c>
-      <c r="P46" s="232">
+      <c r="P46" s="233">
         <f>SUM(P32-G46)</f>
         <v/>
       </c>
-      <c r="Q46" s="232">
+      <c r="Q46" s="233">
         <f>SUM(Q32-H46)</f>
         <v/>
       </c>
-      <c r="R46" s="232">
+      <c r="R46" s="233">
         <f>SUM(R32-I46)</f>
         <v/>
       </c>
-      <c r="S46" s="232">
+      <c r="S46" s="233">
         <f>SUM(S32-J46)</f>
         <v/>
       </c>
-      <c r="T46" s="233">
+      <c r="T46" s="234">
         <f>SUM(T32-K46)</f>
         <v/>
       </c>
@@ -5957,48 +5957,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X46" s="234" t="n"/>
-      <c r="Y46" s="235" t="n"/>
-      <c r="Z46" s="235" t="n"/>
-      <c r="AA46" s="235" t="n"/>
-      <c r="AB46" s="235" t="n"/>
-      <c r="AC46" s="235" t="n"/>
-      <c r="AD46" s="235" t="n"/>
-      <c r="AE46" s="235" t="n"/>
-      <c r="AF46" s="236" t="n"/>
-      <c r="AG46" s="231">
+      <c r="X46" s="235" t="n"/>
+      <c r="Y46" s="236" t="n"/>
+      <c r="Z46" s="236" t="n"/>
+      <c r="AA46" s="236" t="n"/>
+      <c r="AB46" s="236" t="n"/>
+      <c r="AC46" s="236" t="n"/>
+      <c r="AD46" s="236" t="n"/>
+      <c r="AE46" s="236" t="n"/>
+      <c r="AF46" s="237" t="n"/>
+      <c r="AG46" s="232">
         <f>SUM(AG32-X46)</f>
         <v/>
       </c>
-      <c r="AH46" s="232">
+      <c r="AH46" s="233">
         <f>SUM(AH32-Y46)</f>
         <v/>
       </c>
-      <c r="AI46" s="232">
+      <c r="AI46" s="233">
         <f>SUM(AI32-Z46)</f>
         <v/>
       </c>
-      <c r="AJ46" s="232">
+      <c r="AJ46" s="233">
         <f>SUM(AJ32-AA46)</f>
         <v/>
       </c>
-      <c r="AK46" s="232">
+      <c r="AK46" s="233">
         <f>SUM(AK32-AB46)</f>
         <v/>
       </c>
-      <c r="AL46" s="232">
+      <c r="AL46" s="233">
         <f>SUM(AL32-AC46)</f>
         <v/>
       </c>
-      <c r="AM46" s="232">
+      <c r="AM46" s="233">
         <f>SUM(AM32-AD46)</f>
         <v/>
       </c>
-      <c r="AN46" s="232">
+      <c r="AN46" s="233">
         <f>SUM(AN32-AE46)</f>
         <v/>
       </c>
-      <c r="AO46" s="233">
+      <c r="AO46" s="234">
         <f>SUM(AO32-AF46)</f>
         <v/>
       </c>
@@ -6023,39 +6023,39 @@
       <c r="I47" s="215" t="n"/>
       <c r="J47" s="215" t="n"/>
       <c r="K47" s="216" t="n"/>
-      <c r="L47" s="231">
+      <c r="L47" s="232">
         <f>SUM(L33-C47)</f>
         <v/>
       </c>
-      <c r="M47" s="232">
+      <c r="M47" s="233">
         <f>SUM(M33-D47)</f>
         <v/>
       </c>
-      <c r="N47" s="232">
+      <c r="N47" s="233">
         <f>SUM(N33-E47)</f>
         <v/>
       </c>
-      <c r="O47" s="232">
+      <c r="O47" s="233">
         <f>SUM(O33-F47)</f>
         <v/>
       </c>
-      <c r="P47" s="232">
+      <c r="P47" s="233">
         <f>SUM(P33-G47)</f>
         <v/>
       </c>
-      <c r="Q47" s="232">
+      <c r="Q47" s="233">
         <f>SUM(Q33-H47)</f>
         <v/>
       </c>
-      <c r="R47" s="232">
+      <c r="R47" s="233">
         <f>SUM(R33-I47)</f>
         <v/>
       </c>
-      <c r="S47" s="232">
+      <c r="S47" s="233">
         <f>SUM(S33-J47)</f>
         <v/>
       </c>
-      <c r="T47" s="233">
+      <c r="T47" s="234">
         <f>SUM(T33-K47)</f>
         <v/>
       </c>
@@ -6069,48 +6069,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X47" s="234" t="n"/>
-      <c r="Y47" s="235" t="n"/>
-      <c r="Z47" s="235" t="n"/>
-      <c r="AA47" s="235" t="n"/>
-      <c r="AB47" s="235" t="n"/>
-      <c r="AC47" s="235" t="n"/>
-      <c r="AD47" s="235" t="n"/>
-      <c r="AE47" s="235" t="n"/>
-      <c r="AF47" s="236" t="n"/>
-      <c r="AG47" s="231">
+      <c r="X47" s="235" t="n"/>
+      <c r="Y47" s="236" t="n"/>
+      <c r="Z47" s="236" t="n"/>
+      <c r="AA47" s="236" t="n"/>
+      <c r="AB47" s="236" t="n"/>
+      <c r="AC47" s="236" t="n"/>
+      <c r="AD47" s="236" t="n"/>
+      <c r="AE47" s="236" t="n"/>
+      <c r="AF47" s="237" t="n"/>
+      <c r="AG47" s="232">
         <f>SUM(AG33-X47)</f>
         <v/>
       </c>
-      <c r="AH47" s="232">
+      <c r="AH47" s="233">
         <f>SUM(AH33-Y47)</f>
         <v/>
       </c>
-      <c r="AI47" s="232">
+      <c r="AI47" s="233">
         <f>SUM(AI33-Z47)</f>
         <v/>
       </c>
-      <c r="AJ47" s="232">
+      <c r="AJ47" s="233">
         <f>SUM(AJ33-AA47)</f>
         <v/>
       </c>
-      <c r="AK47" s="232">
+      <c r="AK47" s="233">
         <f>SUM(AK33-AB47)</f>
         <v/>
       </c>
-      <c r="AL47" s="232">
+      <c r="AL47" s="233">
         <f>SUM(AL33-AC47)</f>
         <v/>
       </c>
-      <c r="AM47" s="232">
+      <c r="AM47" s="233">
         <f>SUM(AM33-AD47)</f>
         <v/>
       </c>
-      <c r="AN47" s="232">
+      <c r="AN47" s="233">
         <f>SUM(AN33-AE47)</f>
         <v/>
       </c>
-      <c r="AO47" s="233">
+      <c r="AO47" s="234">
         <f>SUM(AO33-AF47)</f>
         <v/>
       </c>
@@ -6126,48 +6126,48 @@
           <t>ICD</t>
         </is>
       </c>
-      <c r="C48" s="234" t="n"/>
-      <c r="D48" s="235" t="n"/>
-      <c r="E48" s="235" t="n"/>
-      <c r="F48" s="235" t="n"/>
-      <c r="G48" s="235" t="n"/>
-      <c r="H48" s="235" t="n"/>
-      <c r="I48" s="235" t="n"/>
-      <c r="J48" s="235" t="n"/>
-      <c r="K48" s="236" t="n"/>
-      <c r="L48" s="231">
+      <c r="C48" s="235" t="n"/>
+      <c r="D48" s="236" t="n"/>
+      <c r="E48" s="236" t="n"/>
+      <c r="F48" s="236" t="n"/>
+      <c r="G48" s="236" t="n"/>
+      <c r="H48" s="236" t="n"/>
+      <c r="I48" s="236" t="n"/>
+      <c r="J48" s="236" t="n"/>
+      <c r="K48" s="237" t="n"/>
+      <c r="L48" s="232">
         <f>SUM(L34-C48)</f>
         <v/>
       </c>
-      <c r="M48" s="232">
+      <c r="M48" s="233">
         <f>SUM(M34-D48)</f>
         <v/>
       </c>
-      <c r="N48" s="232">
+      <c r="N48" s="233">
         <f>SUM(N34-E48)</f>
         <v/>
       </c>
-      <c r="O48" s="232">
+      <c r="O48" s="233">
         <f>SUM(O34-F48)</f>
         <v/>
       </c>
-      <c r="P48" s="232">
+      <c r="P48" s="233">
         <f>SUM(P34-G48)</f>
         <v/>
       </c>
-      <c r="Q48" s="232">
+      <c r="Q48" s="233">
         <f>SUM(Q34-H48)</f>
         <v/>
       </c>
-      <c r="R48" s="232">
+      <c r="R48" s="233">
         <f>SUM(R34-I48)</f>
         <v/>
       </c>
-      <c r="S48" s="232">
+      <c r="S48" s="233">
         <f>SUM(S34-J48)</f>
         <v/>
       </c>
-      <c r="T48" s="233">
+      <c r="T48" s="234">
         <f>SUM(T34-K48)</f>
         <v/>
       </c>
@@ -6181,48 +6181,48 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="X48" s="234" t="n"/>
-      <c r="Y48" s="235" t="n"/>
-      <c r="Z48" s="235" t="n"/>
-      <c r="AA48" s="235" t="n"/>
-      <c r="AB48" s="235" t="n"/>
-      <c r="AC48" s="235" t="n"/>
-      <c r="AD48" s="235" t="n"/>
-      <c r="AE48" s="235" t="n"/>
-      <c r="AF48" s="236" t="n"/>
-      <c r="AG48" s="231">
+      <c r="X48" s="235" t="n"/>
+      <c r="Y48" s="236" t="n"/>
+      <c r="Z48" s="236" t="n"/>
+      <c r="AA48" s="236" t="n"/>
+      <c r="AB48" s="236" t="n"/>
+      <c r="AC48" s="236" t="n"/>
+      <c r="AD48" s="236" t="n"/>
+      <c r="AE48" s="236" t="n"/>
+      <c r="AF48" s="237" t="n"/>
+      <c r="AG48" s="232">
         <f>SUM(AG34-X48)</f>
         <v/>
       </c>
-      <c r="AH48" s="232">
+      <c r="AH48" s="233">
         <f>SUM(AH34-Y48)</f>
         <v/>
       </c>
-      <c r="AI48" s="232">
+      <c r="AI48" s="233">
         <f>SUM(AI34-Z48)</f>
         <v/>
       </c>
-      <c r="AJ48" s="232">
+      <c r="AJ48" s="233">
         <f>SUM(AJ34-AA48)</f>
         <v/>
       </c>
-      <c r="AK48" s="232">
+      <c r="AK48" s="233">
         <f>SUM(AK34-AB48)</f>
         <v/>
       </c>
-      <c r="AL48" s="232">
+      <c r="AL48" s="233">
         <f>SUM(AL34-AC48)</f>
         <v/>
       </c>
-      <c r="AM48" s="232">
+      <c r="AM48" s="233">
         <f>SUM(AM34-AD48)</f>
         <v/>
       </c>
-      <c r="AN48" s="232">
+      <c r="AN48" s="233">
         <f>SUM(AN34-AE48)</f>
         <v/>
       </c>
-      <c r="AO48" s="233">
+      <c r="AO48" s="234">
         <f>SUM(AO34-AF48)</f>
         <v/>
       </c>
@@ -6238,52 +6238,48 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C49" s="237" t="n">
-        <v>110</v>
-      </c>
+      <c r="C49" s="238" t="n"/>
       <c r="D49" s="223" t="n"/>
-      <c r="E49" s="223" t="n">
-        <v>64</v>
-      </c>
+      <c r="E49" s="223" t="n"/>
       <c r="F49" s="223" t="n"/>
       <c r="G49" s="223" t="n"/>
       <c r="H49" s="223" t="n"/>
       <c r="I49" s="223" t="n"/>
       <c r="J49" s="223" t="n"/>
-      <c r="K49" s="238" t="n"/>
-      <c r="L49" s="239">
+      <c r="K49" s="239" t="n"/>
+      <c r="L49" s="240">
         <f>SUM(L35-C49)</f>
         <v/>
       </c>
-      <c r="M49" s="240">
+      <c r="M49" s="241">
         <f>SUM(M35-D49)</f>
         <v/>
       </c>
-      <c r="N49" s="240">
+      <c r="N49" s="241">
         <f>SUM(N35-E49)</f>
         <v/>
       </c>
-      <c r="O49" s="240">
+      <c r="O49" s="241">
         <f>SUM(O35-F49)</f>
         <v/>
       </c>
-      <c r="P49" s="240">
+      <c r="P49" s="241">
         <f>SUM(P35-G49)</f>
         <v/>
       </c>
-      <c r="Q49" s="240">
+      <c r="Q49" s="241">
         <f>SUM(Q35-H49)</f>
         <v/>
       </c>
-      <c r="R49" s="240">
+      <c r="R49" s="241">
         <f>SUM(R35-I49)</f>
         <v/>
       </c>
-      <c r="S49" s="240">
+      <c r="S49" s="241">
         <f>SUM(S35-J49)</f>
         <v/>
       </c>
-      <c r="T49" s="241">
+      <c r="T49" s="242">
         <f>SUM(T35-K49)</f>
         <v/>
       </c>
@@ -6297,56 +6293,48 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X49" s="237" t="n">
-        <v>101</v>
-      </c>
+      <c r="X49" s="238" t="n"/>
       <c r="Y49" s="223" t="n"/>
-      <c r="Z49" s="223" t="n">
-        <v>83</v>
-      </c>
-      <c r="AA49" s="223" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB49" s="223" t="n">
-        <v>21</v>
-      </c>
+      <c r="Z49" s="223" t="n"/>
+      <c r="AA49" s="223" t="n"/>
+      <c r="AB49" s="223" t="n"/>
       <c r="AC49" s="223" t="n"/>
       <c r="AD49" s="223" t="n"/>
       <c r="AE49" s="223" t="n"/>
-      <c r="AF49" s="238" t="n"/>
-      <c r="AG49" s="239">
+      <c r="AF49" s="239" t="n"/>
+      <c r="AG49" s="240">
         <f>SUM(AG35-X49)</f>
         <v/>
       </c>
-      <c r="AH49" s="240">
+      <c r="AH49" s="241">
         <f>SUM(AH35-Y49)</f>
         <v/>
       </c>
-      <c r="AI49" s="240">
+      <c r="AI49" s="241">
         <f>SUM(AI35-Z49)</f>
         <v/>
       </c>
-      <c r="AJ49" s="240">
+      <c r="AJ49" s="241">
         <f>SUM(AJ35-AA49)</f>
         <v/>
       </c>
-      <c r="AK49" s="240">
+      <c r="AK49" s="241">
         <f>SUM(AK35-AB49)</f>
         <v/>
       </c>
-      <c r="AL49" s="240">
+      <c r="AL49" s="241">
         <f>SUM(AL35-AC49)</f>
         <v/>
       </c>
-      <c r="AM49" s="240">
+      <c r="AM49" s="241">
         <f>SUM(AM35-AD49)</f>
         <v/>
       </c>
-      <c r="AN49" s="240">
+      <c r="AN49" s="241">
         <f>SUM(AN35-AE49)</f>
         <v/>
       </c>
-      <c r="AO49" s="241">
+      <c r="AO49" s="242">
         <f>SUM(AO35-AF49)</f>
         <v/>
       </c>
@@ -6362,58 +6350,48 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C50" s="237" t="n">
-        <v>151</v>
-      </c>
-      <c r="D50" s="223" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="223" t="n">
-        <v>145</v>
-      </c>
-      <c r="F50" s="223" t="n">
-        <v>6</v>
-      </c>
-      <c r="G50" s="223" t="n">
-        <v>42</v>
-      </c>
+      <c r="C50" s="238" t="n"/>
+      <c r="D50" s="223" t="n"/>
+      <c r="E50" s="223" t="n"/>
+      <c r="F50" s="223" t="n"/>
+      <c r="G50" s="223" t="n"/>
       <c r="H50" s="223" t="n"/>
       <c r="I50" s="223" t="n"/>
       <c r="J50" s="223" t="n"/>
-      <c r="K50" s="238" t="n"/>
-      <c r="L50" s="239">
+      <c r="K50" s="239" t="n"/>
+      <c r="L50" s="240">
         <f>SUM(L36-C50)</f>
         <v/>
       </c>
-      <c r="M50" s="240">
+      <c r="M50" s="241">
         <f>SUM(M36-D50)</f>
         <v/>
       </c>
-      <c r="N50" s="240">
+      <c r="N50" s="241">
         <f>SUM(N36-E50)</f>
         <v/>
       </c>
-      <c r="O50" s="240">
+      <c r="O50" s="241">
         <f>SUM(O36-F50)</f>
         <v/>
       </c>
-      <c r="P50" s="249">
+      <c r="P50" s="243">
         <f>SUM(P36-G50)</f>
         <v/>
       </c>
-      <c r="Q50" s="240">
+      <c r="Q50" s="241">
         <f>SUM(Q36-H50)</f>
         <v/>
       </c>
-      <c r="R50" s="240">
+      <c r="R50" s="241">
         <f>SUM(R36-I50)</f>
         <v/>
       </c>
-      <c r="S50" s="240">
+      <c r="S50" s="241">
         <f>SUM(S36-J50)</f>
         <v/>
       </c>
-      <c r="T50" s="241">
+      <c r="T50" s="242">
         <f>SUM(T36-K50)</f>
         <v/>
       </c>
@@ -6427,52 +6405,48 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X50" s="237" t="n">
-        <v>11</v>
-      </c>
+      <c r="X50" s="238" t="n"/>
       <c r="Y50" s="223" t="n"/>
-      <c r="Z50" s="223" t="n">
-        <v>11</v>
-      </c>
+      <c r="Z50" s="223" t="n"/>
       <c r="AA50" s="223" t="n"/>
       <c r="AB50" s="223" t="n"/>
       <c r="AC50" s="223" t="n"/>
       <c r="AD50" s="223" t="n"/>
       <c r="AE50" s="223" t="n"/>
-      <c r="AF50" s="238" t="n"/>
-      <c r="AG50" s="239">
+      <c r="AF50" s="239" t="n"/>
+      <c r="AG50" s="240">
         <f>SUM(AG36-X50)</f>
         <v/>
       </c>
-      <c r="AH50" s="240">
+      <c r="AH50" s="241">
         <f>SUM(AH36-Y50)</f>
         <v/>
       </c>
-      <c r="AI50" s="240">
+      <c r="AI50" s="241">
         <f>SUM(AI36-Z50)</f>
         <v/>
       </c>
-      <c r="AJ50" s="240">
+      <c r="AJ50" s="241">
         <f>SUM(AJ36-AA50)</f>
         <v/>
       </c>
-      <c r="AK50" s="240">
+      <c r="AK50" s="241">
         <f>SUM(AK36-AB50)</f>
         <v/>
       </c>
-      <c r="AL50" s="240">
+      <c r="AL50" s="241">
         <f>SUM(AL36-AC50)</f>
         <v/>
       </c>
-      <c r="AM50" s="240">
+      <c r="AM50" s="241">
         <f>SUM(AM36-AD50)</f>
         <v/>
       </c>
-      <c r="AN50" s="240">
+      <c r="AN50" s="241">
         <f>SUM(AN36-AE50)</f>
         <v/>
       </c>
-      <c r="AO50" s="241">
+      <c r="AO50" s="242">
         <f>SUM(AO36-AF50)</f>
         <v/>
       </c>
@@ -6489,39 +6463,39 @@
       <c r="I51" s="28" t="n"/>
       <c r="J51" s="28" t="n"/>
       <c r="K51" s="42" t="n"/>
-      <c r="L51" s="242">
+      <c r="L51" s="244">
         <f>SUM(L37-C51)</f>
         <v/>
       </c>
-      <c r="M51" s="243">
+      <c r="M51" s="245">
         <f>SUM(M37-D51)</f>
         <v/>
       </c>
-      <c r="N51" s="243">
+      <c r="N51" s="245">
         <f>SUM(N37-E51)</f>
         <v/>
       </c>
-      <c r="O51" s="243">
+      <c r="O51" s="245">
         <f>SUM(O37-F51)</f>
         <v/>
       </c>
-      <c r="P51" s="243">
+      <c r="P51" s="245">
         <f>SUM(P37-G51)</f>
         <v/>
       </c>
-      <c r="Q51" s="243">
+      <c r="Q51" s="245">
         <f>SUM(Q37-H51)</f>
         <v/>
       </c>
-      <c r="R51" s="243">
+      <c r="R51" s="245">
         <f>SUM(R37-I51)</f>
         <v/>
       </c>
-      <c r="S51" s="243">
+      <c r="S51" s="245">
         <f>SUM(S37-J51)</f>
         <v/>
       </c>
-      <c r="T51" s="244">
+      <c r="T51" s="246">
         <f>SUM(T37-K51)</f>
         <v/>
       </c>
@@ -6535,52 +6509,48 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X51" s="237" t="n">
-        <v>193</v>
-      </c>
+      <c r="X51" s="238" t="n"/>
       <c r="Y51" s="223" t="n"/>
-      <c r="Z51" s="223" t="n">
-        <v>190</v>
-      </c>
+      <c r="Z51" s="223" t="n"/>
       <c r="AA51" s="223" t="n"/>
       <c r="AB51" s="223" t="n"/>
       <c r="AC51" s="223" t="n"/>
       <c r="AD51" s="223" t="n"/>
       <c r="AE51" s="223" t="n"/>
-      <c r="AF51" s="238" t="n"/>
-      <c r="AG51" s="239">
+      <c r="AF51" s="239" t="n"/>
+      <c r="AG51" s="240">
         <f>SUM(AG37-X51)</f>
         <v/>
       </c>
-      <c r="AH51" s="240">
+      <c r="AH51" s="241">
         <f>SUM(AH37-Y51)</f>
         <v/>
       </c>
-      <c r="AI51" s="240">
+      <c r="AI51" s="241">
         <f>SUM(AI37-Z51)</f>
         <v/>
       </c>
-      <c r="AJ51" s="240">
+      <c r="AJ51" s="241">
         <f>SUM(AJ37-AA51)</f>
         <v/>
       </c>
-      <c r="AK51" s="240">
+      <c r="AK51" s="241">
         <f>SUM(AK37-AB51)</f>
         <v/>
       </c>
-      <c r="AL51" s="240">
+      <c r="AL51" s="241">
         <f>SUM(AL37-AC51)</f>
         <v/>
       </c>
-      <c r="AM51" s="240">
+      <c r="AM51" s="241">
         <f>SUM(AM37-AD51)</f>
         <v/>
       </c>
-      <c r="AN51" s="240">
+      <c r="AN51" s="241">
         <f>SUM(AN37-AE51)</f>
         <v/>
       </c>
-      <c r="AO51" s="241">
+      <c r="AO51" s="242">
         <f>SUM(AO37-AF51)</f>
         <v/>
       </c>
@@ -6597,39 +6567,39 @@
       <c r="I52" s="28" t="n"/>
       <c r="J52" s="28" t="n"/>
       <c r="K52" s="42" t="n"/>
-      <c r="L52" s="242">
+      <c r="L52" s="244">
         <f>SUM(L38-C52)</f>
         <v/>
       </c>
-      <c r="M52" s="243">
+      <c r="M52" s="245">
         <f>SUM(M38-D52)</f>
         <v/>
       </c>
-      <c r="N52" s="243">
+      <c r="N52" s="245">
         <f>SUM(N38-E52)</f>
         <v/>
       </c>
-      <c r="O52" s="243">
+      <c r="O52" s="245">
         <f>SUM(O38-F52)</f>
         <v/>
       </c>
-      <c r="P52" s="243">
+      <c r="P52" s="245">
         <f>SUM(P38-G52)</f>
         <v/>
       </c>
-      <c r="Q52" s="243">
+      <c r="Q52" s="245">
         <f>SUM(Q38-H52)</f>
         <v/>
       </c>
-      <c r="R52" s="243">
+      <c r="R52" s="245">
         <f>SUM(R38-I52)</f>
         <v/>
       </c>
-      <c r="S52" s="243">
+      <c r="S52" s="245">
         <f>SUM(S38-J52)</f>
         <v/>
       </c>
-      <c r="T52" s="244">
+      <c r="T52" s="246">
         <f>SUM(T38-K52)</f>
         <v/>
       </c>
@@ -6644,39 +6614,39 @@
       <c r="AD52" s="49" t="n"/>
       <c r="AE52" s="49" t="n"/>
       <c r="AF52" s="82" t="n"/>
-      <c r="AG52" s="242">
+      <c r="AG52" s="244">
         <f>SUM(AG38-X52)</f>
         <v/>
       </c>
-      <c r="AH52" s="243">
+      <c r="AH52" s="245">
         <f>SUM(AH38-Y52)</f>
         <v/>
       </c>
-      <c r="AI52" s="243">
+      <c r="AI52" s="245">
         <f>SUM(AI38-Z52)</f>
         <v/>
       </c>
-      <c r="AJ52" s="243">
+      <c r="AJ52" s="245">
         <f>SUM(AJ38-AA52)</f>
         <v/>
       </c>
-      <c r="AK52" s="243">
+      <c r="AK52" s="245">
         <f>SUM(AK38-AB52)</f>
         <v/>
       </c>
-      <c r="AL52" s="243">
+      <c r="AL52" s="245">
         <f>SUM(AL38-AC52)</f>
         <v/>
       </c>
-      <c r="AM52" s="243">
+      <c r="AM52" s="245">
         <f>SUM(AM38-AD52)</f>
         <v/>
       </c>
-      <c r="AN52" s="243">
+      <c r="AN52" s="245">
         <f>SUM(AN38-AE52)</f>
         <v/>
       </c>
-      <c r="AO52" s="244">
+      <c r="AO52" s="246">
         <f>SUM(AO38-AF52)</f>
         <v/>
       </c>
@@ -6693,39 +6663,39 @@
       <c r="I53" s="28" t="n"/>
       <c r="J53" s="28" t="n"/>
       <c r="K53" s="42" t="n"/>
-      <c r="L53" s="242">
+      <c r="L53" s="244">
         <f>SUM(L39-C53)</f>
         <v/>
       </c>
-      <c r="M53" s="243">
+      <c r="M53" s="245">
         <f>SUM(M39-D53)</f>
         <v/>
       </c>
-      <c r="N53" s="243">
+      <c r="N53" s="245">
         <f>SUM(N39-E53)</f>
         <v/>
       </c>
-      <c r="O53" s="243">
+      <c r="O53" s="245">
         <f>SUM(O39-F53)</f>
         <v/>
       </c>
-      <c r="P53" s="243">
+      <c r="P53" s="245">
         <f>SUM(P39-G53)</f>
         <v/>
       </c>
-      <c r="Q53" s="243">
+      <c r="Q53" s="245">
         <f>SUM(Q39-H53)</f>
         <v/>
       </c>
-      <c r="R53" s="243">
+      <c r="R53" s="245">
         <f>SUM(R39-I53)</f>
         <v/>
       </c>
-      <c r="S53" s="243">
+      <c r="S53" s="245">
         <f>SUM(S39-J53)</f>
         <v/>
       </c>
-      <c r="T53" s="244">
+      <c r="T53" s="246">
         <f>SUM(T39-K53)</f>
         <v/>
       </c>
@@ -6740,39 +6710,39 @@
       <c r="AD53" s="49" t="n"/>
       <c r="AE53" s="49" t="n"/>
       <c r="AF53" s="82" t="n"/>
-      <c r="AG53" s="242">
+      <c r="AG53" s="244">
         <f>SUM(AG39-X53)</f>
         <v/>
       </c>
-      <c r="AH53" s="243">
+      <c r="AH53" s="245">
         <f>SUM(AH39-Y53)</f>
         <v/>
       </c>
-      <c r="AI53" s="243">
+      <c r="AI53" s="245">
         <f>SUM(AI39-Z53)</f>
         <v/>
       </c>
-      <c r="AJ53" s="243">
+      <c r="AJ53" s="245">
         <f>SUM(AJ39-AA53)</f>
         <v/>
       </c>
-      <c r="AK53" s="243">
+      <c r="AK53" s="245">
         <f>SUM(AK39-AB53)</f>
         <v/>
       </c>
-      <c r="AL53" s="243">
+      <c r="AL53" s="245">
         <f>SUM(AL39-AC53)</f>
         <v/>
       </c>
-      <c r="AM53" s="243">
+      <c r="AM53" s="245">
         <f>SUM(AM39-AD53)</f>
         <v/>
       </c>
-      <c r="AN53" s="243">
+      <c r="AN53" s="245">
         <f>SUM(AN39-AE53)</f>
         <v/>
       </c>
-      <c r="AO53" s="244">
+      <c r="AO53" s="246">
         <f>SUM(AO39-AF53)</f>
         <v/>
       </c>
@@ -6793,39 +6763,39 @@
       <c r="I54" s="85" t="n"/>
       <c r="J54" s="85" t="n"/>
       <c r="K54" s="86" t="n"/>
-      <c r="L54" s="245">
+      <c r="L54" s="247">
         <f>SUM(L40-C54)</f>
         <v/>
       </c>
-      <c r="M54" s="246">
+      <c r="M54" s="248">
         <f>SUM(M40-D54)</f>
         <v/>
       </c>
-      <c r="N54" s="246">
+      <c r="N54" s="248">
         <f>SUM(N40-E54)</f>
         <v/>
       </c>
-      <c r="O54" s="246">
+      <c r="O54" s="248">
         <f>SUM(O40-F54)</f>
         <v/>
       </c>
-      <c r="P54" s="246">
+      <c r="P54" s="248">
         <f>SUM(P40-G54)</f>
         <v/>
       </c>
-      <c r="Q54" s="246">
+      <c r="Q54" s="248">
         <f>SUM(Q40-H54)</f>
         <v/>
       </c>
-      <c r="R54" s="246">
+      <c r="R54" s="248">
         <f>SUM(R40-I54)</f>
         <v/>
       </c>
-      <c r="S54" s="246">
+      <c r="S54" s="248">
         <f>SUM(S40-J54)</f>
         <v/>
       </c>
-      <c r="T54" s="247">
+      <c r="T54" s="249">
         <f>SUM(T40-K54)</f>
         <v/>
       </c>
@@ -6845,39 +6815,39 @@
       <c r="AD54" s="85" t="n"/>
       <c r="AE54" s="85" t="n"/>
       <c r="AF54" s="86" t="n"/>
-      <c r="AG54" s="242">
+      <c r="AG54" s="244">
         <f>SUM(AG40-X54)</f>
         <v/>
       </c>
-      <c r="AH54" s="243">
+      <c r="AH54" s="245">
         <f>SUM(AH40-Y54)</f>
         <v/>
       </c>
-      <c r="AI54" s="243">
+      <c r="AI54" s="245">
         <f>SUM(AI40-Z54)</f>
         <v/>
       </c>
-      <c r="AJ54" s="243">
+      <c r="AJ54" s="245">
         <f>SUM(AJ40-AA54)</f>
         <v/>
       </c>
-      <c r="AK54" s="243">
+      <c r="AK54" s="245">
         <f>SUM(AK40-AB54)</f>
         <v/>
       </c>
-      <c r="AL54" s="243">
+      <c r="AL54" s="245">
         <f>SUM(AL40-AC54)</f>
         <v/>
       </c>
-      <c r="AM54" s="243">
+      <c r="AM54" s="245">
         <f>SUM(AM40-AD54)</f>
         <v/>
       </c>
-      <c r="AN54" s="243">
+      <c r="AN54" s="245">
         <f>SUM(AN40-AE54)</f>
         <v/>
       </c>
-      <c r="AO54" s="244">
+      <c r="AO54" s="246">
         <f>SUM(AO40-AF54)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Friday's 2nd STOCK BALANCE END WK slot uses WK3RD booking, not blank
Per sirichai: after WK1ST absorbs WK1+WK2 on a Friday, the second slot
should show the following week (WK3RD, Mon-Sun the week after next)
instead of sitting empty - keeps two forward-looking windows always
visible. Corrects 2026-09-18 (28/09-04/10 window, cross-checked against
the raw booking file).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock Daily 2026-09-18.xlsx
+++ b/Stock Daily 2026-09-18.xlsx
@@ -1049,7 +1049,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1758,6 +1758,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="10" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5536,7 +5539,7 @@
       <c r="H43" s="188" t="n"/>
       <c r="I43" s="197" t="inlineStr">
         <is>
-          <t>21-27/09/2026</t>
+          <t>28/09-04/10/2026</t>
         </is>
       </c>
       <c r="J43" s="187" t="n"/>
@@ -5573,7 +5576,7 @@
       <c r="AC43" s="188" t="n"/>
       <c r="AD43" s="197" t="inlineStr">
         <is>
-          <t>21-27/09/2026</t>
+          <t>28/09-04/10/2026</t>
         </is>
       </c>
       <c r="AE43" s="187" t="n"/>
@@ -5790,9 +5793,13 @@
           <t>TERMINAL</t>
         </is>
       </c>
-      <c r="C45" s="206" t="n"/>
+      <c r="C45" s="206" t="n">
+        <v>7</v>
+      </c>
       <c r="D45" s="207" t="n"/>
-      <c r="E45" s="207" t="n"/>
+      <c r="E45" s="207" t="n">
+        <v>14</v>
+      </c>
       <c r="F45" s="207" t="n"/>
       <c r="G45" s="207" t="n"/>
       <c r="H45" s="207" t="n"/>
@@ -5807,7 +5814,7 @@
         <f>SUM(M31-D45)</f>
         <v/>
       </c>
-      <c r="N45" s="226">
+      <c r="N45" s="250">
         <f>SUM(N31-E45)</f>
         <v/>
       </c>
@@ -6238,9 +6245,13 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C49" s="238" t="n"/>
+      <c r="C49" s="238" t="n">
+        <v>89</v>
+      </c>
       <c r="D49" s="223" t="n"/>
-      <c r="E49" s="223" t="n"/>
+      <c r="E49" s="223" t="n">
+        <v>40</v>
+      </c>
       <c r="F49" s="223" t="n"/>
       <c r="G49" s="223" t="n"/>
       <c r="H49" s="223" t="n"/>
@@ -6293,11 +6304,19 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X49" s="238" t="n"/>
+      <c r="X49" s="238" t="n">
+        <v>53</v>
+      </c>
       <c r="Y49" s="223" t="n"/>
-      <c r="Z49" s="223" t="n"/>
-      <c r="AA49" s="223" t="n"/>
-      <c r="AB49" s="223" t="n"/>
+      <c r="Z49" s="223" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA49" s="223" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB49" s="223" t="n">
+        <v>7</v>
+      </c>
       <c r="AC49" s="223" t="n"/>
       <c r="AD49" s="223" t="n"/>
       <c r="AE49" s="223" t="n"/>
@@ -6350,11 +6369,19 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="C50" s="238" t="n"/>
+      <c r="C50" s="238" t="n">
+        <v>66</v>
+      </c>
       <c r="D50" s="223" t="n"/>
-      <c r="E50" s="223" t="n"/>
-      <c r="F50" s="223" t="n"/>
-      <c r="G50" s="223" t="n"/>
+      <c r="E50" s="223" t="n">
+        <v>29</v>
+      </c>
+      <c r="F50" s="223" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" s="223" t="n">
+        <v>3</v>
+      </c>
       <c r="H50" s="223" t="n"/>
       <c r="I50" s="223" t="n"/>
       <c r="J50" s="223" t="n"/>
@@ -6407,7 +6434,9 @@
       </c>
       <c r="X50" s="238" t="n"/>
       <c r="Y50" s="223" t="n"/>
-      <c r="Z50" s="223" t="n"/>
+      <c r="Z50" s="223" t="n">
+        <v>17</v>
+      </c>
       <c r="AA50" s="223" t="n"/>
       <c r="AB50" s="223" t="n"/>
       <c r="AC50" s="223" t="n"/>
@@ -6509,15 +6538,21 @@
           <t>DEPOT</t>
         </is>
       </c>
-      <c r="X51" s="238" t="n"/>
+      <c r="X51" s="238" t="n">
+        <v>114</v>
+      </c>
       <c r="Y51" s="223" t="n"/>
-      <c r="Z51" s="223" t="n"/>
+      <c r="Z51" s="223" t="n">
+        <v>61</v>
+      </c>
       <c r="AA51" s="223" t="n"/>
       <c r="AB51" s="223" t="n"/>
       <c r="AC51" s="223" t="n"/>
       <c r="AD51" s="223" t="n"/>
       <c r="AE51" s="223" t="n"/>
-      <c r="AF51" s="239" t="n"/>
+      <c r="AF51" s="239" t="n">
+        <v>1</v>
+      </c>
       <c r="AG51" s="240">
         <f>SUM(AG37-X51)</f>
         <v/>
@@ -7615,39 +7650,39 @@
           <t>E/P In (this week)</t>
         </is>
       </c>
-      <c r="C4" s="250">
+      <c r="C4" s="251">
         <f>Daily!L14</f>
         <v/>
       </c>
-      <c r="D4" s="250">
+      <c r="D4" s="251">
         <f>Daily!M14</f>
         <v/>
       </c>
-      <c r="E4" s="250">
+      <c r="E4" s="251">
         <f>Daily!N14</f>
         <v/>
       </c>
-      <c r="F4" s="250">
+      <c r="F4" s="251">
         <f>Daily!O14</f>
         <v/>
       </c>
-      <c r="G4" s="250">
+      <c r="G4" s="251">
         <f>Daily!P14</f>
         <v/>
       </c>
-      <c r="H4" s="250">
+      <c r="H4" s="251">
         <f>Daily!Q14</f>
         <v/>
       </c>
-      <c r="I4" s="250">
+      <c r="I4" s="251">
         <f>Daily!R14</f>
         <v/>
       </c>
-      <c r="J4" s="250">
+      <c r="J4" s="251">
         <f>Daily!S14</f>
         <v/>
       </c>
-      <c r="K4" s="250">
+      <c r="K4" s="251">
         <f>Daily!T14</f>
         <v/>
       </c>
@@ -7682,39 +7717,39 @@
           <t>INBOUND MT RETURN</t>
         </is>
       </c>
-      <c r="C7" s="251">
+      <c r="C7" s="252">
         <f>Daily!C15</f>
         <v/>
       </c>
-      <c r="D7" s="251">
+      <c r="D7" s="252">
         <f>Daily!D15</f>
         <v/>
       </c>
-      <c r="E7" s="251">
+      <c r="E7" s="252">
         <f>Daily!E15</f>
         <v/>
       </c>
-      <c r="F7" s="251">
+      <c r="F7" s="252">
         <f>Daily!F15</f>
         <v/>
       </c>
-      <c r="G7" s="251">
+      <c r="G7" s="252">
         <f>Daily!G15</f>
         <v/>
       </c>
-      <c r="H7" s="251">
+      <c r="H7" s="252">
         <f>Daily!H15</f>
         <v/>
       </c>
-      <c r="I7" s="251">
+      <c r="I7" s="252">
         <f>Daily!I15</f>
         <v/>
       </c>
-      <c r="J7" s="251">
+      <c r="J7" s="252">
         <f>Daily!J15</f>
         <v/>
       </c>
-      <c r="K7" s="251">
+      <c r="K7" s="252">
         <f>Daily!K15</f>
         <v/>
       </c>
@@ -7725,39 +7760,39 @@
           <t>Booking(This week)</t>
         </is>
       </c>
-      <c r="C8" s="250">
+      <c r="C8" s="251">
         <f>Daily!C41</f>
         <v/>
       </c>
-      <c r="D8" s="250">
+      <c r="D8" s="251">
         <f>Daily!D41</f>
         <v/>
       </c>
-      <c r="E8" s="250">
+      <c r="E8" s="251">
         <f>Daily!E41</f>
         <v/>
       </c>
-      <c r="F8" s="250">
+      <c r="F8" s="251">
         <f>Daily!F41</f>
         <v/>
       </c>
-      <c r="G8" s="250">
+      <c r="G8" s="251">
         <f>Daily!G41</f>
         <v/>
       </c>
-      <c r="H8" s="250">
+      <c r="H8" s="251">
         <f>Daily!H41</f>
         <v/>
       </c>
-      <c r="I8" s="250">
+      <c r="I8" s="251">
         <f>Daily!I41</f>
         <v/>
       </c>
-      <c r="J8" s="250">
+      <c r="J8" s="251">
         <f>Daily!J41</f>
         <v/>
       </c>
-      <c r="K8" s="250">
+      <c r="K8" s="251">
         <f>Daily!K41</f>
         <v/>
       </c>
@@ -7772,39 +7807,39 @@
           <t>Booking(Next week)</t>
         </is>
       </c>
-      <c r="C9" s="252">
+      <c r="C9" s="253">
         <f>Daily!C55</f>
         <v/>
       </c>
-      <c r="D9" s="252">
+      <c r="D9" s="253">
         <f>Daily!D55</f>
         <v/>
       </c>
-      <c r="E9" s="252">
+      <c r="E9" s="253">
         <f>Daily!E55</f>
         <v/>
       </c>
-      <c r="F9" s="252">
+      <c r="F9" s="253">
         <f>Daily!F55</f>
         <v/>
       </c>
-      <c r="G9" s="252">
+      <c r="G9" s="253">
         <f>Daily!G55</f>
         <v/>
       </c>
-      <c r="H9" s="252">
+      <c r="H9" s="253">
         <f>Daily!H55</f>
         <v/>
       </c>
-      <c r="I9" s="252">
+      <c r="I9" s="253">
         <f>Daily!I55</f>
         <v/>
       </c>
-      <c r="J9" s="252">
+      <c r="J9" s="253">
         <f>Daily!J55</f>
         <v/>
       </c>
-      <c r="K9" s="252">
+      <c r="K9" s="253">
         <f>Daily!K55</f>
         <v/>
       </c>
@@ -7819,39 +7854,39 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="C10" s="253">
+      <c r="C10" s="254">
         <f>SUM(C3+C4+C5+C6+C7-C8-C9)</f>
         <v/>
       </c>
-      <c r="D10" s="253">
+      <c r="D10" s="254">
         <f>SUM(D3+D4+D5+D6+D7-D8-D9)</f>
         <v/>
       </c>
-      <c r="E10" s="253">
+      <c r="E10" s="254">
         <f>SUM(E3+E4+E5+E6+E7-E8-E9)</f>
         <v/>
       </c>
-      <c r="F10" s="253">
+      <c r="F10" s="254">
         <f>SUM(F3+F4+F5+F6+F7-F8-F9)</f>
         <v/>
       </c>
-      <c r="G10" s="254">
+      <c r="G10" s="255">
         <f>SUM(G3+G4+G5+G6+G7-G8-G9)</f>
         <v/>
       </c>
-      <c r="H10" s="253">
+      <c r="H10" s="254">
         <f>SUM(H3+H4+H5+H6+H7-H8-H9)</f>
         <v/>
       </c>
-      <c r="I10" s="253">
+      <c r="I10" s="254">
         <f>SUM(I3+I4+I5+I6+I7-I8-I9)</f>
         <v/>
       </c>
-      <c r="J10" s="253">
+      <c r="J10" s="254">
         <f>SUM(J3+J4+J5+J6+J7-J8-J9)</f>
         <v/>
       </c>
-      <c r="K10" s="253">
+      <c r="K10" s="254">
         <f>SUM(K3+K4+K5+K6+K7-K8-K9)</f>
         <v/>
       </c>
@@ -7985,39 +8020,39 @@
           <t>E/P In (this week)</t>
         </is>
       </c>
-      <c r="C15" s="250">
+      <c r="C15" s="251">
         <f>Daily!AG14</f>
         <v/>
       </c>
-      <c r="D15" s="250">
+      <c r="D15" s="251">
         <f>Daily!AH14</f>
         <v/>
       </c>
-      <c r="E15" s="250">
+      <c r="E15" s="251">
         <f>Daily!AI14</f>
         <v/>
       </c>
-      <c r="F15" s="250">
+      <c r="F15" s="251">
         <f>Daily!AJ14</f>
         <v/>
       </c>
-      <c r="G15" s="250">
+      <c r="G15" s="251">
         <f>Daily!AK14</f>
         <v/>
       </c>
-      <c r="H15" s="250">
+      <c r="H15" s="251">
         <f>Daily!AL14</f>
         <v/>
       </c>
-      <c r="I15" s="250">
+      <c r="I15" s="251">
         <f>Daily!AM14</f>
         <v/>
       </c>
-      <c r="J15" s="250">
+      <c r="J15" s="251">
         <f>Daily!AN14</f>
         <v/>
       </c>
-      <c r="K15" s="250">
+      <c r="K15" s="251">
         <f>Daily!AO14</f>
         <v/>
       </c>
@@ -8052,39 +8087,39 @@
           <t>INBOUND MT RETURN</t>
         </is>
       </c>
-      <c r="C18" s="251">
+      <c r="C18" s="252">
         <f>Daily!X15</f>
         <v/>
       </c>
-      <c r="D18" s="251">
+      <c r="D18" s="252">
         <f>Daily!Y15</f>
         <v/>
       </c>
-      <c r="E18" s="251">
+      <c r="E18" s="252">
         <f>Daily!Z15</f>
         <v/>
       </c>
-      <c r="F18" s="251">
+      <c r="F18" s="252">
         <f>Daily!AA15</f>
         <v/>
       </c>
-      <c r="G18" s="251">
+      <c r="G18" s="252">
         <f>Daily!AB15</f>
         <v/>
       </c>
-      <c r="H18" s="251">
+      <c r="H18" s="252">
         <f>Daily!AC15</f>
         <v/>
       </c>
-      <c r="I18" s="251">
+      <c r="I18" s="252">
         <f>Daily!AD15</f>
         <v/>
       </c>
-      <c r="J18" s="251">
+      <c r="J18" s="252">
         <f>Daily!AE15</f>
         <v/>
       </c>
-      <c r="K18" s="251">
+      <c r="K18" s="252">
         <f>Daily!AF15</f>
         <v/>
       </c>
@@ -8095,39 +8130,39 @@
           <t>Booking(This week)</t>
         </is>
       </c>
-      <c r="C19" s="252">
+      <c r="C19" s="253">
         <f>Daily!X41</f>
         <v/>
       </c>
-      <c r="D19" s="252">
+      <c r="D19" s="253">
         <f>Daily!Y41</f>
         <v/>
       </c>
-      <c r="E19" s="252">
+      <c r="E19" s="253">
         <f>Daily!Z41</f>
         <v/>
       </c>
-      <c r="F19" s="252">
+      <c r="F19" s="253">
         <f>Daily!AA41</f>
         <v/>
       </c>
-      <c r="G19" s="252">
+      <c r="G19" s="253">
         <f>Daily!AB41</f>
         <v/>
       </c>
-      <c r="H19" s="252">
+      <c r="H19" s="253">
         <f>Daily!AC41</f>
         <v/>
       </c>
-      <c r="I19" s="255">
+      <c r="I19" s="256">
         <f>Daily!AD41</f>
         <v/>
       </c>
-      <c r="J19" s="255">
+      <c r="J19" s="256">
         <f>Daily!AE41</f>
         <v/>
       </c>
-      <c r="K19" s="252">
+      <c r="K19" s="253">
         <f>Daily!AF41</f>
         <v/>
       </c>
@@ -8142,39 +8177,39 @@
           <t>Booking(Next week)</t>
         </is>
       </c>
-      <c r="C20" s="252">
+      <c r="C20" s="253">
         <f>Daily!X55</f>
         <v/>
       </c>
-      <c r="D20" s="252">
+      <c r="D20" s="253">
         <f>Daily!Y55</f>
         <v/>
       </c>
-      <c r="E20" s="252">
+      <c r="E20" s="253">
         <f>Daily!Z55</f>
         <v/>
       </c>
-      <c r="F20" s="252">
+      <c r="F20" s="253">
         <f>Daily!AA55</f>
         <v/>
       </c>
-      <c r="G20" s="252">
+      <c r="G20" s="253">
         <f>Daily!AB55</f>
         <v/>
       </c>
-      <c r="H20" s="252">
+      <c r="H20" s="253">
         <f>Daily!AC55</f>
         <v/>
       </c>
-      <c r="I20" s="252">
+      <c r="I20" s="253">
         <f>Daily!AD55</f>
         <v/>
       </c>
-      <c r="J20" s="252">
+      <c r="J20" s="253">
         <f>Daily!AE55</f>
         <v/>
       </c>
-      <c r="K20" s="252">
+      <c r="K20" s="253">
         <f>Daily!AF55</f>
         <v/>
       </c>
@@ -8189,39 +8224,39 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="C21" s="253">
+      <c r="C21" s="254">
         <f>SUM(C14+C15+C16+C17+C18-C19-C20)</f>
         <v/>
       </c>
-      <c r="D21" s="253">
+      <c r="D21" s="254">
         <f>SUM(D14+D15+D16+D17+D18-D19-D20)</f>
         <v/>
       </c>
-      <c r="E21" s="253">
+      <c r="E21" s="254">
         <f>SUM(E14+E15+E16+E17+E18-E19-E20)</f>
         <v/>
       </c>
-      <c r="F21" s="253">
+      <c r="F21" s="254">
         <f>SUM(F14+F15+F16+F17+F18-F19-F20)</f>
         <v/>
       </c>
-      <c r="G21" s="253">
+      <c r="G21" s="254">
         <f>SUM(G14+G15+G16+G17+G18-G19-G20)</f>
         <v/>
       </c>
-      <c r="H21" s="253">
+      <c r="H21" s="254">
         <f>SUM(H14+H15+H16+H17+H18-H19-H20)</f>
         <v/>
       </c>
-      <c r="I21" s="253">
+      <c r="I21" s="254">
         <f>SUM(I14+I15+I16+I17+I18-I19-I20)</f>
         <v/>
       </c>
-      <c r="J21" s="253">
+      <c r="J21" s="254">
         <f>SUM(J14+J15+J16+J17+J18-J19-J20)</f>
         <v/>
       </c>
-      <c r="K21" s="253">
+      <c r="K21" s="254">
         <f>SUM(K14+K15+K16+K17+K18-K19-K20)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix REPO (E/P) going blank: EMPTY.xls schema changed to per-container
Since 2026-09-18 the EP2/EMPTY file is a raw per-container list (one row
per container, 'Type Size' column holding the type as text) instead of
the original one-row-per-vessel format with count columns (22GP, 42GP,
...). repo_ep_totals() summed those count columns unconditionally, which
no longer exist, so every total came out 0 and the whole row went blank.

Now detects which schema is present and counts rows (per-container) or
sums columns (aggregated) accordingly - same 'match by content' approach
already used for the booking file's schema changes. Verified against the
raw file's own row counts (THLCH: 162x22GP, 59x45GP) and confirmed live
on the dashboard.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock Daily 2026-09-18.xlsx
+++ b/Stock Daily 2026-09-18.xlsx
@@ -3335,9 +3335,13 @@
       <c r="AD14" s="26" t="n"/>
       <c r="AE14" s="26" t="n"/>
       <c r="AF14" s="27" t="n"/>
-      <c r="AG14" s="50" t="n"/>
+      <c r="AG14" s="50" t="n">
+        <v>162</v>
+      </c>
       <c r="AH14" s="51" t="n"/>
-      <c r="AI14" s="51" t="n"/>
+      <c r="AI14" s="51" t="n">
+        <v>59</v>
+      </c>
       <c r="AJ14" s="51" t="n"/>
       <c r="AK14" s="51" t="n"/>
       <c r="AL14" s="51" t="n"/>

</xml_diff>